<commit_message>
lots of stuff i can't even
</commit_message>
<xml_diff>
--- a/data/Experiment/Raw/StomatalDensity.xlsx
+++ b/data/Experiment/Raw/StomatalDensity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fernbromley/Desktop/SeedlingMortality/data/Experiment/Raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967ED056-FC8F-9443-B141-EC87796E49A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EF2985D-383D-0640-A889-57FED081192B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15640" yWindow="5900" windowWidth="13120" windowHeight="12060" xr2:uid="{CA551DF1-0ED1-674A-8F89-05216640288A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="244">
   <si>
     <t>PIPO1</t>
   </si>
@@ -1172,7 +1172,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F958DE17-0E59-E849-A835-10176DABDFD5}">
-  <dimension ref="A1:D147"/>
+  <dimension ref="A1:D153"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -1248,7 +1248,7 @@
         <v>25</v>
       </c>
       <c r="D5">
-        <f t="shared" ref="D5:D147" si="0">C5/B5</f>
+        <f t="shared" ref="D5:D153" si="0">C5/B5</f>
         <v>59.382422802850357</v>
       </c>
     </row>
@@ -3083,7 +3083,7 @@
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A128" s="2" t="s">
+      <c r="A128" s="5" t="s">
         <v>43</v>
       </c>
       <c r="B128">
@@ -3098,7 +3098,7 @@
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A129" s="2" t="s">
+      <c r="A129" s="5" t="s">
         <v>43</v>
       </c>
       <c r="B129">
@@ -3113,7 +3113,7 @@
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A130" s="2" t="s">
+      <c r="A130" s="5" t="s">
         <v>43</v>
       </c>
       <c r="B130">
@@ -3128,89 +3128,143 @@
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A131" s="2" t="s">
+      <c r="A131" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D131" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+      <c r="B131">
+        <v>1.083</v>
+      </c>
+      <c r="C131">
+        <v>70</v>
+      </c>
+      <c r="D131">
+        <f t="shared" si="0"/>
+        <v>64.635272391505083</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A132" s="2" t="s">
+      <c r="A132" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B132">
+        <v>0.45500000000000002</v>
+      </c>
+      <c r="C132">
+        <v>30</v>
+      </c>
+      <c r="D132">
+        <f t="shared" ref="D132" si="43">C132/B132</f>
+        <v>65.934065934065927</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A133" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B133">
+        <v>0.249</v>
+      </c>
+      <c r="C133">
+        <v>11</v>
+      </c>
+      <c r="D133">
+        <f t="shared" si="0"/>
+        <v>44.176706827309239</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A134" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D132" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A133" s="2" t="s">
+      <c r="B134">
+        <v>0.76900000000000002</v>
+      </c>
+      <c r="C134">
+        <v>38</v>
+      </c>
+      <c r="D134">
+        <f t="shared" si="0"/>
+        <v>49.414824447334198</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A135" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B135">
+        <v>0.76900000000000002</v>
+      </c>
+      <c r="C135">
+        <v>40</v>
+      </c>
+      <c r="D135">
+        <f t="shared" ref="D135" si="44">C135/B135</f>
+        <v>52.015604681404419</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A136" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B136">
+        <v>0.20799999999999999</v>
+      </c>
+      <c r="C136">
+        <v>10</v>
+      </c>
+      <c r="D136">
+        <f t="shared" si="0"/>
+        <v>48.07692307692308</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A137" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D133" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A134" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D134" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A135" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D135" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A136" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D136" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A137" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D137" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+      <c r="B137">
+        <v>1.659</v>
+      </c>
+      <c r="C137">
+        <v>88</v>
+      </c>
+      <c r="D137">
+        <f t="shared" si="0"/>
+        <v>53.044002411091014</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A138" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D138" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+      <c r="A138" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B138">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="C138">
+        <v>44</v>
+      </c>
+      <c r="D138">
+        <f t="shared" ref="D138" si="45">C138/B138</f>
+        <v>75.862068965517253</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A139" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D139" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+      <c r="A139" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B139">
+        <v>1.3680000000000001</v>
+      </c>
+      <c r="C139">
+        <v>73</v>
+      </c>
+      <c r="D139">
+        <f t="shared" si="0"/>
+        <v>53.362573099415201</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A140" s="2" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="D140" t="e">
         <f t="shared" si="0"/>
@@ -3219,7 +3273,7 @@
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A141" s="2" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="D141" t="e">
         <f t="shared" si="0"/>
@@ -3228,7 +3282,7 @@
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A142" s="2" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D142" t="e">
         <f t="shared" si="0"/>
@@ -3237,7 +3291,7 @@
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A143" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D143" t="e">
         <f t="shared" si="0"/>
@@ -3246,7 +3300,7 @@
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A144" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D144" t="e">
         <f t="shared" si="0"/>
@@ -3255,7 +3309,7 @@
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A145" s="2" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D145" t="e">
         <f t="shared" si="0"/>
@@ -3264,7 +3318,7 @@
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A146" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D146" t="e">
         <f t="shared" si="0"/>
@@ -3273,9 +3327,63 @@
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A147" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D147" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A148" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D148" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A149" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D149" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A150" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D150" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A151" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D151" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A152" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D152" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A153" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D147" t="e">
+      <c r="D153" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>

</xml_diff>